<commit_message>
Enhance Excel extraction agent with new features and configurations
- Updated `.env.example` to include additional environment variables for n8n runners and Excel tools, improving configuration options.
- Modified `docker-compose.yml` to integrate n8n runners as a separate service with enhanced resource management and security settings.
- Enhanced `README.md` with updated architecture details and instructions for using the new agent tool request format.
- Introduced a new context seeder for static Excel-agent operating guidance, ensuring deterministic behavior in the FastAPI service.
- Improved session management and validation logic in the FastAPI application to handle concurrent requests more effectively.

These changes significantly enhance the functionality, security, and usability of the Excel extraction agent.
</commit_message>
<xml_diff>
--- a/excel-agent-tools/tests/fixtures/complex/06_blank_line_and_total_row.xlsx
+++ b/excel-agent-tools/tests/fixtures/complex/06_blank_line_and_total_row.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -486,52 +486,52 @@
         <v>21500</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>CC-30</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Support</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>12000</v>
-      </c>
-      <c r="D5" t="n">
-        <v>9000</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>CC-40</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>HR</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>8000</v>
-      </c>
-      <c r="D6" t="n">
-        <v>7800</v>
-      </c>
-    </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>CC-30</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Support</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>12000</v>
+      </c>
+      <c r="D7" t="n">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>CC-40</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>8000</v>
+      </c>
+      <c r="D10" t="n">
+        <v>7800</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C7" t="n">
+      <c r="C11" t="n">
         <v>90000</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D11" t="n">
         <v>86300</v>
       </c>
     </row>

</xml_diff>